<commit_message>
feat: integrate runtime audio volume control
</commit_message>
<xml_diff>
--- a/99_Doc/voice_checkpoint_resouce_map.xlsx
+++ b/99_Doc/voice_checkpoint_resouce_map.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="24090" windowHeight="15300" activeTab="1"/>
+    <workbookView windowWidth="24090" windowHeight="15300"/>
   </bookViews>
   <sheets>
     <sheet name="引脚分配" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="421">
   <si>
     <t>AT32F435VGT7 MCU资源分配表</t>
   </si>
@@ -869,7 +869,7 @@
     <t>BOARD_GPIO_KEY1 (33)</t>
   </si>
   <si>
-    <t>板载按键，低有效</t>
+    <t>板载按键，低有效,对应板子丝印SW2</t>
   </si>
   <si>
     <t>PE1</t>
@@ -881,6 +881,9 @@
     <t>BOARD_GPIO_KEY2 (34)</t>
   </si>
   <si>
+    <t>板载按键，低有效，对应板子丝印SW3</t>
+  </si>
+  <si>
     <t>PE2</t>
   </si>
   <si>
@@ -890,6 +893,9 @@
     <t>BOARD_GPIO_KEY3 (35)</t>
   </si>
   <si>
+    <t>板载按键，低有效，对应板子丝印SW4</t>
+  </si>
+  <si>
     <t>PE3</t>
   </si>
   <si>
@@ -897,6 +903,9 @@
   </si>
   <si>
     <t>BOARD_GPIO_KEY4 (36)</t>
+  </si>
+  <si>
+    <t>板载按键，低有效，对应板子丝印SW5</t>
   </si>
   <si>
     <t>PE4</t>
@@ -5390,7 +5399,7 @@
         <v>281</v>
       </c>
       <c r="L66" s="16" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="M66" s="16" t="s">
         <v>24</v>
@@ -5404,10 +5413,10 @@
         <v>63</v>
       </c>
       <c r="B67" s="15" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C67" s="15" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D67" s="15" t="s">
         <v>132</v>
@@ -5431,10 +5440,10 @@
         <v>22</v>
       </c>
       <c r="K67" s="15" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="L67" s="16" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="M67" s="16" t="s">
         <v>24</v>
@@ -5448,10 +5457,10 @@
         <v>64</v>
       </c>
       <c r="B68" s="15" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C68" s="15" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D68" s="15" t="s">
         <v>132</v>
@@ -5475,10 +5484,10 @@
         <v>22</v>
       </c>
       <c r="K68" s="15" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="L68" s="16" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="M68" s="16" t="s">
         <v>24</v>
@@ -5492,10 +5501,10 @@
         <v>65</v>
       </c>
       <c r="B69" s="15" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C69" s="15" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="D69" s="15" t="s">
         <v>132</v>
@@ -5519,10 +5528,10 @@
         <v>22</v>
       </c>
       <c r="K69" s="15" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="L69" s="16" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="M69" s="16" t="s">
         <v>24</v>
@@ -5536,10 +5545,10 @@
         <v>66</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C70" s="15" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="D70" s="15" t="s">
         <v>52</v>
@@ -5563,10 +5572,10 @@
         <v>54</v>
       </c>
       <c r="K70" s="15" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="L70" s="16" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="M70" s="16" t="s">
         <v>24</v>
@@ -5580,10 +5589,10 @@
         <v>67</v>
       </c>
       <c r="B71" s="15" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C71" s="15" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="D71" s="15" t="s">
         <v>52</v>
@@ -5607,10 +5616,10 @@
         <v>127</v>
       </c>
       <c r="K71" s="15" t="s">
+        <v>301</v>
+      </c>
+      <c r="L71" s="16" t="s">
         <v>298</v>
-      </c>
-      <c r="L71" s="16" t="s">
-        <v>295</v>
       </c>
       <c r="M71" s="16" t="s">
         <v>24</v>
@@ -5624,10 +5633,10 @@
         <v>68</v>
       </c>
       <c r="B72" s="15" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C72" s="15" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D72" s="15" t="s">
         <v>52</v>
@@ -5651,7 +5660,7 @@
         <v>54</v>
       </c>
       <c r="K72" s="15" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="L72" s="16" t="s">
         <v>86</v>
@@ -5668,10 +5677,10 @@
         <v>69</v>
       </c>
       <c r="B73" s="15" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C73" s="15" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="D73" s="15" t="s">
         <v>52</v>
@@ -5695,7 +5704,7 @@
         <v>54</v>
       </c>
       <c r="K73" s="15" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="L73" s="16" t="s">
         <v>86</v>
@@ -5712,10 +5721,10 @@
         <v>70</v>
       </c>
       <c r="B74" s="15" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="C74" s="15" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="D74" s="15" t="s">
         <v>52</v>
@@ -5742,7 +5751,7 @@
         <v>22</v>
       </c>
       <c r="L74" s="16" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="M74" s="16" t="s">
         <v>24</v>
@@ -5756,10 +5765,10 @@
         <v>71</v>
       </c>
       <c r="B75" s="15" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C75" s="15" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D75" s="15" t="s">
         <v>32</v>
@@ -5768,7 +5777,7 @@
         <v>33</v>
       </c>
       <c r="F75" s="15" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="G75" s="15" t="s">
         <v>71</v>
@@ -5786,7 +5795,7 @@
         <v>22</v>
       </c>
       <c r="L75" s="16" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="M75" s="16" t="s">
         <v>24</v>
@@ -5800,10 +5809,10 @@
         <v>72</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C76" s="15" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D76" s="15" t="s">
         <v>32</v>
@@ -5812,10 +5821,10 @@
         <v>18</v>
       </c>
       <c r="F76" s="15" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="G76" s="15" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="H76" s="15" t="s">
         <v>99</v>
@@ -5830,7 +5839,7 @@
         <v>22</v>
       </c>
       <c r="L76" s="16" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="M76" s="16" t="s">
         <v>24</v>
@@ -5844,10 +5853,10 @@
         <v>73</v>
       </c>
       <c r="B77" s="15" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C77" s="15" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="D77" s="15" t="s">
         <v>52</v>
@@ -5871,10 +5880,10 @@
         <v>127</v>
       </c>
       <c r="K77" s="15" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="L77" s="16" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="M77" s="16" t="s">
         <v>24</v>
@@ -5888,10 +5897,10 @@
         <v>74</v>
       </c>
       <c r="B78" s="15" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C78" s="15" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="D78" s="15" t="s">
         <v>52</v>
@@ -5915,10 +5924,10 @@
         <v>127</v>
       </c>
       <c r="K78" s="15" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="L78" s="16" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="M78" s="16" t="s">
         <v>24</v>
@@ -5932,10 +5941,10 @@
         <v>75</v>
       </c>
       <c r="B79" s="15" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C79" s="15" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="D79" s="15" t="s">
         <v>52</v>
@@ -5959,10 +5968,10 @@
         <v>127</v>
       </c>
       <c r="K79" s="15" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="L79" s="16" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="M79" s="16" t="s">
         <v>24</v>
@@ -5976,10 +5985,10 @@
         <v>76</v>
       </c>
       <c r="B80" s="15" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="C80" s="15" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D80" s="15" t="s">
         <v>52</v>
@@ -6003,10 +6012,10 @@
         <v>127</v>
       </c>
       <c r="K80" s="15" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="L80" s="16" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="M80" s="16" t="s">
         <v>24</v>
@@ -6020,10 +6029,10 @@
         <v>77</v>
       </c>
       <c r="B81" s="15" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="C81" s="15" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="D81" s="15" t="s">
         <v>32</v>
@@ -6035,7 +6044,7 @@
         <v>218</v>
       </c>
       <c r="G81" s="15" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="H81" s="15" t="s">
         <v>21</v>
@@ -6050,7 +6059,7 @@
         <v>22</v>
       </c>
       <c r="L81" s="16" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="M81" s="16" t="s">
         <v>24</v>
@@ -6064,7 +6073,7 @@
         <v>78</v>
       </c>
       <c r="B82" s="15" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="C82" s="15" t="s">
         <v>192</v>
@@ -6136,7 +6145,7 @@
   <sheetData>
     <row r="1" ht="62" customHeight="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6148,25 +6157,25 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>14</v>
@@ -6174,28 +6183,28 @@
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:8">
       <c r="A3" s="3" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:8">
@@ -6203,65 +6212,65 @@
         <v>70</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>354</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>355</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:8">
       <c r="A5" s="3" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:8">
       <c r="A6" s="3" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>21</v>
@@ -6270,10 +6279,10 @@
         <v>24</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:8">
@@ -6281,25 +6290,25 @@
         <v>46</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:8">
@@ -6307,13 +6316,13 @@
         <v>92</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>21</v>
@@ -6322,10 +6331,10 @@
         <v>24</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:8">
@@ -6333,25 +6342,25 @@
         <v>60</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:8">
@@ -6359,39 +6368,39 @@
         <v>34</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1" spans="1:8">
       <c r="A11" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>21</v>
@@ -6400,10 +6409,10 @@
         <v>24</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1" spans="1:8">
@@ -6411,13 +6420,13 @@
         <v>19</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>21</v>
@@ -6426,10 +6435,10 @@
         <v>24</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1" spans="1:8">
@@ -6437,25 +6446,25 @@
         <v>154</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1" spans="1:8">
@@ -6463,13 +6472,13 @@
         <v>53</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>21</v>
@@ -6478,24 +6487,24 @@
         <v>24</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="15" ht="34" customHeight="1" spans="1:8">
       <c r="A15" s="3" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>22</v>
@@ -6504,10 +6513,10 @@
         <v>24</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test: add HUB GPIO level verification
</commit_message>
<xml_diff>
--- a/99_Doc/voice_checkpoint_resouce_map.xlsx
+++ b/99_Doc/voice_checkpoint_resouce_map.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="24090" windowHeight="15300"/>
+    <workbookView windowWidth="26180" windowHeight="15300"/>
   </bookViews>
   <sheets>
     <sheet name="引脚分配" sheetId="1" r:id="rId1"/>
@@ -302,7 +302,7 @@
     <t>RS485_RXEN</t>
   </si>
   <si>
-    <t>RS485收发方向控制；驱动=中等；未纳入Board GPIO资源表</t>
+    <t>RS485收发方向控制；驱动=中等；未纳入Board GPIO资源表,高电平-TX模式，低电平-RX模式</t>
   </si>
   <si>
     <t>PA15</t>
@@ -3208,7 +3208,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" ht="38" spans="1:14">
+    <row r="17" ht="57" spans="1:14">
       <c r="A17" s="15">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
feat: integrate HUB display voice presentation
Add HUB12 scrolling display and PC9 power control, coordinate captions with voice LEDs through a presentation app, and refresh clangd data after successful builds.
</commit_message>
<xml_diff>
--- a/99_Doc/voice_checkpoint_resouce_map.xlsx
+++ b/99_Doc/voice_checkpoint_resouce_map.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="422">
   <si>
     <t>AT32F435VGT7 MCU资源分配表</t>
   </si>
@@ -611,6 +611,237 @@
     <t>PC6</t>
   </si>
   <si>
+    <t>HUB_OE245</t>
+  </si>
+  <si>
+    <t>还未绑定</t>
+  </si>
+  <si>
+    <t>HUB显示接口；驱动=增强</t>
+  </si>
+  <si>
+    <t>wk_gpio.c</t>
+  </si>
+  <si>
+    <t>PC7</t>
+  </si>
+  <si>
+    <t>LED_OUT_B</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_LED_OUT_B (2)</t>
+  </si>
+  <si>
+    <t>外部双色LED控制；驱动=中等</t>
+  </si>
+  <si>
+    <t>PC8</t>
+  </si>
+  <si>
+    <t>LED_OUT_R</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_LED_OUT_R (3)</t>
+  </si>
+  <si>
+    <t>PC9</t>
+  </si>
+  <si>
+    <t>LED_POWER_CS</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_LED_POWER_CS (4)</t>
+  </si>
+  <si>
+    <t>LED电源/片选控制；驱动=中等，高电平关闭，低电平打开</t>
+  </si>
+  <si>
+    <t>PC10</t>
+  </si>
+  <si>
+    <t>PIR_IN</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_PIR_IN (30)</t>
+  </si>
+  <si>
+    <t>PIR人体感应</t>
+  </si>
+  <si>
+    <t>PC11</t>
+  </si>
+  <si>
+    <t>QSPI1_WS</t>
+  </si>
+  <si>
+    <t>AF9 / CS</t>
+  </si>
+  <si>
+    <t>QSPI1 CS；驱动=增强</t>
+  </si>
+  <si>
+    <t>PC12</t>
+  </si>
+  <si>
+    <t>EEPROM_SDA</t>
+  </si>
+  <si>
+    <t>I2C2/EEPROM</t>
+  </si>
+  <si>
+    <t>AF4 / SDA</t>
+  </si>
+  <si>
+    <t>开漏</t>
+  </si>
+  <si>
+    <t>I2C2/EEPROM SDA；驱动=中等</t>
+  </si>
+  <si>
+    <t>at32f435_437_wk_config.h；wk_i2c.c</t>
+  </si>
+  <si>
+    <t>PC13</t>
+  </si>
+  <si>
+    <t>SDIO2_TFCD</t>
+  </si>
+  <si>
+    <t>TF卡插入检测；未纳入Board GPIO资源表</t>
+  </si>
+  <si>
+    <t>PD0</t>
+  </si>
+  <si>
+    <t>HUB_A</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_A (15)</t>
+  </si>
+  <si>
+    <t>PD1</t>
+  </si>
+  <si>
+    <t>HUB_B</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_B (16)</t>
+  </si>
+  <si>
+    <t>PD2</t>
+  </si>
+  <si>
+    <t>HUB_C</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_C (17)</t>
+  </si>
+  <si>
+    <t>PD3</t>
+  </si>
+  <si>
+    <t>HUB_D</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_D (18)</t>
+  </si>
+  <si>
+    <t>PD4</t>
+  </si>
+  <si>
+    <t>HUB_E</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_E (19)</t>
+  </si>
+  <si>
+    <t>PD5</t>
+  </si>
+  <si>
+    <t>HUB_LAT</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_LAT (20)</t>
+  </si>
+  <si>
+    <t>HUB显示接口；驱动=中等</t>
+  </si>
+  <si>
+    <t>PD6</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_OE245 (21)</t>
+  </si>
+  <si>
+    <t>PD7</t>
+  </si>
+  <si>
+    <t>ALARM_IN</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_ALARM_IN (31)</t>
+  </si>
+  <si>
+    <t>紧急喊话/报警接口</t>
+  </si>
+  <si>
+    <t>PD8</t>
+  </si>
+  <si>
+    <t>HUB_R1</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_R1 (22)</t>
+  </si>
+  <si>
+    <t>PD9</t>
+  </si>
+  <si>
+    <t>HUB_G1</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_G1 (23)</t>
+  </si>
+  <si>
+    <t>PD10</t>
+  </si>
+  <si>
+    <t>HUB_B1</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_B1 (24)</t>
+  </si>
+  <si>
+    <t>PD11</t>
+  </si>
+  <si>
+    <t>HUB_R2</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_R2 (25)</t>
+  </si>
+  <si>
+    <t>PD12</t>
+  </si>
+  <si>
+    <t>HUB_G2</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_G2 (26)</t>
+  </si>
+  <si>
+    <t>PD13</t>
+  </si>
+  <si>
+    <t>HUB_B2</t>
+  </si>
+  <si>
+    <t>BOARD_GPIO_HUB_B2 (27)</t>
+  </si>
+  <si>
+    <t>PD14</t>
+  </si>
+  <si>
     <t>未分配</t>
   </si>
   <si>
@@ -621,234 +852,6 @@
   </si>
   <si>
     <t>配置为模拟模式以降低未使用引脚功耗</t>
-  </si>
-  <si>
-    <t>wk_gpio.c</t>
-  </si>
-  <si>
-    <t>PC7</t>
-  </si>
-  <si>
-    <t>LED_OUT_B</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_LED_OUT_B (2)</t>
-  </si>
-  <si>
-    <t>外部双色LED控制；驱动=中等</t>
-  </si>
-  <si>
-    <t>PC8</t>
-  </si>
-  <si>
-    <t>LED_OUT_R</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_LED_OUT_R (3)</t>
-  </si>
-  <si>
-    <t>PC9</t>
-  </si>
-  <si>
-    <t>LED_POWER_CS</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_LED_POWER_CS (4)</t>
-  </si>
-  <si>
-    <t>LED电源/片选控制；驱动=中等</t>
-  </si>
-  <si>
-    <t>PC10</t>
-  </si>
-  <si>
-    <t>PIR_IN</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_PIR_IN (30)</t>
-  </si>
-  <si>
-    <t>PIR人体感应</t>
-  </si>
-  <si>
-    <t>PC11</t>
-  </si>
-  <si>
-    <t>QSPI1_WS</t>
-  </si>
-  <si>
-    <t>AF9 / CS</t>
-  </si>
-  <si>
-    <t>QSPI1 CS；驱动=增强</t>
-  </si>
-  <si>
-    <t>PC12</t>
-  </si>
-  <si>
-    <t>EEPROM_SDA</t>
-  </si>
-  <si>
-    <t>I2C2/EEPROM</t>
-  </si>
-  <si>
-    <t>AF4 / SDA</t>
-  </si>
-  <si>
-    <t>开漏</t>
-  </si>
-  <si>
-    <t>I2C2/EEPROM SDA；驱动=中等</t>
-  </si>
-  <si>
-    <t>at32f435_437_wk_config.h；wk_i2c.c</t>
-  </si>
-  <si>
-    <t>PC13</t>
-  </si>
-  <si>
-    <t>SDIO2_TFCD</t>
-  </si>
-  <si>
-    <t>TF卡插入检测；未纳入Board GPIO资源表</t>
-  </si>
-  <si>
-    <t>PD0</t>
-  </si>
-  <si>
-    <t>HUB_A</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_A (15)</t>
-  </si>
-  <si>
-    <t>HUB显示接口；驱动=增强</t>
-  </si>
-  <si>
-    <t>PD1</t>
-  </si>
-  <si>
-    <t>HUB_B</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_B (16)</t>
-  </si>
-  <si>
-    <t>PD2</t>
-  </si>
-  <si>
-    <t>HUB_C</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_C (17)</t>
-  </si>
-  <si>
-    <t>PD3</t>
-  </si>
-  <si>
-    <t>HUB_D</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_D (18)</t>
-  </si>
-  <si>
-    <t>PD4</t>
-  </si>
-  <si>
-    <t>HUB_E</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_E (19)</t>
-  </si>
-  <si>
-    <t>PD5</t>
-  </si>
-  <si>
-    <t>HUB_LAT</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_LAT (20)</t>
-  </si>
-  <si>
-    <t>HUB显示接口；驱动=中等</t>
-  </si>
-  <si>
-    <t>PD6</t>
-  </si>
-  <si>
-    <t>HUB_OE245</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_OE245 (21)</t>
-  </si>
-  <si>
-    <t>PD7</t>
-  </si>
-  <si>
-    <t>ALARM_IN</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_ALARM_IN (31)</t>
-  </si>
-  <si>
-    <t>紧急喊话/报警接口</t>
-  </si>
-  <si>
-    <t>PD8</t>
-  </si>
-  <si>
-    <t>HUB_R1</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_R1 (22)</t>
-  </si>
-  <si>
-    <t>PD9</t>
-  </si>
-  <si>
-    <t>HUB_G1</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_G1 (23)</t>
-  </si>
-  <si>
-    <t>PD10</t>
-  </si>
-  <si>
-    <t>HUB_B1</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_B1 (24)</t>
-  </si>
-  <si>
-    <t>PD11</t>
-  </si>
-  <si>
-    <t>HUB_R2</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_R2 (25)</t>
-  </si>
-  <si>
-    <t>PD12</t>
-  </si>
-  <si>
-    <t>HUB_G2</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_G2 (26)</t>
-  </si>
-  <si>
-    <t>PD13</t>
-  </si>
-  <si>
-    <t>HUB_B2</t>
-  </si>
-  <si>
-    <t>BOARD_GPIO_HUB_B2 (27)</t>
-  </si>
-  <si>
-    <t>PD14</t>
   </si>
   <si>
     <t>PD15</t>
@@ -4275,37 +4278,37 @@
         <v>192</v>
       </c>
       <c r="D41" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="F41" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="G41" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="H41" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="I41" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="J41" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="K41" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="E41" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="F41" s="15" t="s">
+      <c r="L41" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="G41" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H41" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="I41" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="J41" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="K41" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="L41" s="16" t="s">
+      <c r="M41" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N41" s="16" t="s">
         <v>195</v>
-      </c>
-      <c r="M41" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="N41" s="16" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="42" ht="38" spans="1:14">
@@ -4313,10 +4316,10 @@
         <v>38</v>
       </c>
       <c r="B42" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="C42" s="15" t="s">
         <v>197</v>
-      </c>
-      <c r="C42" s="15" t="s">
-        <v>198</v>
       </c>
       <c r="D42" s="15" t="s">
         <v>52</v>
@@ -4340,10 +4343,10 @@
         <v>54</v>
       </c>
       <c r="K42" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="L42" s="16" t="s">
         <v>199</v>
-      </c>
-      <c r="L42" s="16" t="s">
-        <v>200</v>
       </c>
       <c r="M42" s="16" t="s">
         <v>24</v>
@@ -4357,10 +4360,10 @@
         <v>39</v>
       </c>
       <c r="B43" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="C43" s="15" t="s">
         <v>201</v>
-      </c>
-      <c r="C43" s="15" t="s">
-        <v>202</v>
       </c>
       <c r="D43" s="15" t="s">
         <v>52</v>
@@ -4384,10 +4387,10 @@
         <v>54</v>
       </c>
       <c r="K43" s="15" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L43" s="16" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="M43" s="16" t="s">
         <v>24</v>
@@ -4401,10 +4404,10 @@
         <v>40</v>
       </c>
       <c r="B44" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="C44" s="15" t="s">
         <v>204</v>
-      </c>
-      <c r="C44" s="15" t="s">
-        <v>205</v>
       </c>
       <c r="D44" s="15" t="s">
         <v>52</v>
@@ -4425,13 +4428,13 @@
         <v>36</v>
       </c>
       <c r="J44" s="15" t="s">
-        <v>54</v>
+        <v>127</v>
       </c>
       <c r="K44" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="L44" s="16" t="s">
         <v>206</v>
-      </c>
-      <c r="L44" s="16" t="s">
-        <v>207</v>
       </c>
       <c r="M44" s="16" t="s">
         <v>24</v>
@@ -4445,10 +4448,10 @@
         <v>41</v>
       </c>
       <c r="B45" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="C45" s="15" t="s">
         <v>208</v>
-      </c>
-      <c r="C45" s="15" t="s">
-        <v>209</v>
       </c>
       <c r="D45" s="15" t="s">
         <v>132</v>
@@ -4472,10 +4475,10 @@
         <v>22</v>
       </c>
       <c r="K45" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="L45" s="16" t="s">
         <v>210</v>
-      </c>
-      <c r="L45" s="16" t="s">
-        <v>211</v>
       </c>
       <c r="M45" s="16" t="s">
         <v>24</v>
@@ -4489,10 +4492,10 @@
         <v>42</v>
       </c>
       <c r="B46" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="C46" s="15" t="s">
         <v>212</v>
-      </c>
-      <c r="C46" s="15" t="s">
-        <v>213</v>
       </c>
       <c r="D46" s="15" t="s">
         <v>32</v>
@@ -4504,7 +4507,7 @@
         <v>60</v>
       </c>
       <c r="G46" s="15" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H46" s="15" t="s">
         <v>21</v>
@@ -4519,7 +4522,7 @@
         <v>22</v>
       </c>
       <c r="L46" s="16" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="M46" s="16" t="s">
         <v>24</v>
@@ -4533,10 +4536,10 @@
         <v>43</v>
       </c>
       <c r="B47" s="15" t="s">
+        <v>215</v>
+      </c>
+      <c r="C47" s="15" t="s">
         <v>216</v>
-      </c>
-      <c r="C47" s="15" t="s">
-        <v>217</v>
       </c>
       <c r="D47" s="15" t="s">
         <v>32</v>
@@ -4545,31 +4548,31 @@
         <v>41</v>
       </c>
       <c r="F47" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="G47" s="15" t="s">
         <v>218</v>
       </c>
-      <c r="G47" s="15" t="s">
+      <c r="H47" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="I47" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="H47" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="I47" s="15" t="s">
+      <c r="J47" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="K47" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="L47" s="16" t="s">
         <v>220</v>
       </c>
-      <c r="J47" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="K47" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="L47" s="16" t="s">
+      <c r="M47" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N47" s="16" t="s">
         <v>221</v>
-      </c>
-      <c r="M47" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="N47" s="16" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="48" ht="38" spans="1:14">
@@ -4577,10 +4580,10 @@
         <v>44</v>
       </c>
       <c r="B48" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="C48" s="15" t="s">
         <v>223</v>
-      </c>
-      <c r="C48" s="15" t="s">
-        <v>224</v>
       </c>
       <c r="D48" s="15" t="s">
         <v>132</v>
@@ -4607,7 +4610,7 @@
         <v>22</v>
       </c>
       <c r="L48" s="16" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="M48" s="16" t="s">
         <v>24</v>
@@ -4621,10 +4624,10 @@
         <v>45</v>
       </c>
       <c r="B49" s="15" t="s">
+        <v>225</v>
+      </c>
+      <c r="C49" s="15" t="s">
         <v>226</v>
-      </c>
-      <c r="C49" s="15" t="s">
-        <v>227</v>
       </c>
       <c r="D49" s="15" t="s">
         <v>52</v>
@@ -4648,10 +4651,10 @@
         <v>54</v>
       </c>
       <c r="K49" s="15" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="L49" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M49" s="16" t="s">
         <v>24</v>
@@ -4665,10 +4668,10 @@
         <v>46</v>
       </c>
       <c r="B50" s="15" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D50" s="15" t="s">
         <v>52</v>
@@ -4692,10 +4695,10 @@
         <v>54</v>
       </c>
       <c r="K50" s="15" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="L50" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M50" s="16" t="s">
         <v>24</v>
@@ -4709,10 +4712,10 @@
         <v>47</v>
       </c>
       <c r="B51" s="15" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="D51" s="15" t="s">
         <v>52</v>
@@ -4736,10 +4739,10 @@
         <v>54</v>
       </c>
       <c r="K51" s="15" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L51" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M51" s="16" t="s">
         <v>24</v>
@@ -4753,10 +4756,10 @@
         <v>48</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D52" s="15" t="s">
         <v>52</v>
@@ -4780,10 +4783,10 @@
         <v>54</v>
       </c>
       <c r="K52" s="15" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="L52" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M52" s="16" t="s">
         <v>24</v>
@@ -4797,10 +4800,10 @@
         <v>49</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C53" s="15" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D53" s="15" t="s">
         <v>52</v>
@@ -4824,10 +4827,10 @@
         <v>54</v>
       </c>
       <c r="K53" s="15" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="L53" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M53" s="16" t="s">
         <v>24</v>
@@ -4841,10 +4844,10 @@
         <v>50</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C54" s="15" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D54" s="15" t="s">
         <v>52</v>
@@ -4868,10 +4871,10 @@
         <v>54</v>
       </c>
       <c r="K54" s="15" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="L54" s="16" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="M54" s="16" t="s">
         <v>24</v>
@@ -4885,10 +4888,10 @@
         <v>51</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>247</v>
+        <v>192</v>
       </c>
       <c r="D55" s="15" t="s">
         <v>52</v>
@@ -4912,10 +4915,10 @@
         <v>127</v>
       </c>
       <c r="K55" s="15" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="L55" s="16" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="M55" s="16" t="s">
         <v>24</v>
@@ -4929,10 +4932,10 @@
         <v>52</v>
       </c>
       <c r="B56" s="15" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="C56" s="15" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D56" s="15" t="s">
         <v>132</v>
@@ -4956,10 +4959,10 @@
         <v>22</v>
       </c>
       <c r="K56" s="15" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="L56" s="16" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="M56" s="16" t="s">
         <v>24</v>
@@ -4973,10 +4976,10 @@
         <v>53</v>
       </c>
       <c r="B57" s="15" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C57" s="15" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D57" s="15" t="s">
         <v>52</v>
@@ -5000,10 +5003,10 @@
         <v>54</v>
       </c>
       <c r="K57" s="15" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="L57" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M57" s="16" t="s">
         <v>24</v>
@@ -5017,10 +5020,10 @@
         <v>54</v>
       </c>
       <c r="B58" s="15" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C58" s="15" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="D58" s="15" t="s">
         <v>52</v>
@@ -5044,10 +5047,10 @@
         <v>54</v>
       </c>
       <c r="K58" s="15" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="L58" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M58" s="16" t="s">
         <v>24</v>
@@ -5061,10 +5064,10 @@
         <v>55</v>
       </c>
       <c r="B59" s="15" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C59" s="15" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D59" s="15" t="s">
         <v>52</v>
@@ -5088,10 +5091,10 @@
         <v>54</v>
       </c>
       <c r="K59" s="15" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="L59" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M59" s="16" t="s">
         <v>24</v>
@@ -5105,10 +5108,10 @@
         <v>56</v>
       </c>
       <c r="B60" s="15" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D60" s="15" t="s">
         <v>52</v>
@@ -5132,10 +5135,10 @@
         <v>54</v>
       </c>
       <c r="K60" s="15" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="L60" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M60" s="16" t="s">
         <v>24</v>
@@ -5149,10 +5152,10 @@
         <v>57</v>
       </c>
       <c r="B61" s="15" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C61" s="15" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D61" s="15" t="s">
         <v>52</v>
@@ -5176,10 +5179,10 @@
         <v>54</v>
       </c>
       <c r="K61" s="15" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="L61" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M61" s="16" t="s">
         <v>24</v>
@@ -5193,10 +5196,10 @@
         <v>58</v>
       </c>
       <c r="B62" s="15" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D62" s="15" t="s">
         <v>52</v>
@@ -5220,10 +5223,10 @@
         <v>54</v>
       </c>
       <c r="K62" s="15" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="L62" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M62" s="16" t="s">
         <v>24</v>
@@ -5237,20 +5240,20 @@
         <v>59</v>
       </c>
       <c r="B63" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="C63" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="D63" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="E63" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F63" s="15" t="s">
         <v>271</v>
       </c>
-      <c r="C63" s="15" t="s">
-        <v>192</v>
-      </c>
-      <c r="D63" s="15" t="s">
-        <v>193</v>
-      </c>
-      <c r="E63" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="F63" s="15" t="s">
-        <v>194</v>
-      </c>
       <c r="G63" s="15" t="s">
         <v>22</v>
       </c>
@@ -5267,13 +5270,13 @@
         <v>22</v>
       </c>
       <c r="L63" s="16" t="s">
+        <v>272</v>
+      </c>
+      <c r="M63" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N63" s="16" t="s">
         <v>195</v>
-      </c>
-      <c r="M63" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="N63" s="16" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="64" ht="38" spans="1:14">
@@ -5281,10 +5284,10 @@
         <v>60</v>
       </c>
       <c r="B64" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C64" s="15" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D64" s="15" t="s">
         <v>52</v>
@@ -5308,10 +5311,10 @@
         <v>54</v>
       </c>
       <c r="K64" s="15" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L64" s="16" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="M64" s="16" t="s">
         <v>24</v>
@@ -5325,10 +5328,10 @@
         <v>61</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C65" s="15" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D65" s="15" t="s">
         <v>132</v>
@@ -5352,10 +5355,10 @@
         <v>22</v>
       </c>
       <c r="K65" s="15" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="L65" s="16" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="M65" s="16" t="s">
         <v>24</v>
@@ -5369,10 +5372,10 @@
         <v>62</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C66" s="15" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D66" s="15" t="s">
         <v>132</v>
@@ -5396,10 +5399,10 @@
         <v>22</v>
       </c>
       <c r="K66" s="15" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L66" s="16" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="M66" s="16" t="s">
         <v>24</v>
@@ -5413,10 +5416,10 @@
         <v>63</v>
       </c>
       <c r="B67" s="15" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C67" s="15" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D67" s="15" t="s">
         <v>132</v>
@@ -5440,10 +5443,10 @@
         <v>22</v>
       </c>
       <c r="K67" s="15" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L67" s="16" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="M67" s="16" t="s">
         <v>24</v>
@@ -5457,10 +5460,10 @@
         <v>64</v>
       </c>
       <c r="B68" s="15" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C68" s="15" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D68" s="15" t="s">
         <v>132</v>
@@ -5484,10 +5487,10 @@
         <v>22</v>
       </c>
       <c r="K68" s="15" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L68" s="16" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="M68" s="16" t="s">
         <v>24</v>
@@ -5501,10 +5504,10 @@
         <v>65</v>
       </c>
       <c r="B69" s="15" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C69" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D69" s="15" t="s">
         <v>132</v>
@@ -5528,10 +5531,10 @@
         <v>22</v>
       </c>
       <c r="K69" s="15" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="L69" s="16" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="M69" s="16" t="s">
         <v>24</v>
@@ -5545,10 +5548,10 @@
         <v>66</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C70" s="15" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D70" s="15" t="s">
         <v>52</v>
@@ -5572,10 +5575,10 @@
         <v>54</v>
       </c>
       <c r="K70" s="15" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L70" s="16" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="M70" s="16" t="s">
         <v>24</v>
@@ -5589,10 +5592,10 @@
         <v>67</v>
       </c>
       <c r="B71" s="15" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C71" s="15" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D71" s="15" t="s">
         <v>52</v>
@@ -5616,10 +5619,10 @@
         <v>127</v>
       </c>
       <c r="K71" s="15" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L71" s="16" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="M71" s="16" t="s">
         <v>24</v>
@@ -5633,10 +5636,10 @@
         <v>68</v>
       </c>
       <c r="B72" s="15" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C72" s="15" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D72" s="15" t="s">
         <v>52</v>
@@ -5660,7 +5663,7 @@
         <v>54</v>
       </c>
       <c r="K72" s="15" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L72" s="16" t="s">
         <v>86</v>
@@ -5677,10 +5680,10 @@
         <v>69</v>
       </c>
       <c r="B73" s="15" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C73" s="15" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D73" s="15" t="s">
         <v>52</v>
@@ -5704,7 +5707,7 @@
         <v>54</v>
       </c>
       <c r="K73" s="15" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="L73" s="16" t="s">
         <v>86</v>
@@ -5721,10 +5724,10 @@
         <v>70</v>
       </c>
       <c r="B74" s="15" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C74" s="15" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D74" s="15" t="s">
         <v>52</v>
@@ -5751,7 +5754,7 @@
         <v>22</v>
       </c>
       <c r="L74" s="16" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="M74" s="16" t="s">
         <v>24</v>
@@ -5765,10 +5768,10 @@
         <v>71</v>
       </c>
       <c r="B75" s="15" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C75" s="15" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D75" s="15" t="s">
         <v>32</v>
@@ -5777,7 +5780,7 @@
         <v>33</v>
       </c>
       <c r="F75" s="15" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G75" s="15" t="s">
         <v>71</v>
@@ -5795,7 +5798,7 @@
         <v>22</v>
       </c>
       <c r="L75" s="16" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="M75" s="16" t="s">
         <v>24</v>
@@ -5809,10 +5812,10 @@
         <v>72</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C76" s="15" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D76" s="15" t="s">
         <v>32</v>
@@ -5821,10 +5824,10 @@
         <v>18</v>
       </c>
       <c r="F76" s="15" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G76" s="15" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="H76" s="15" t="s">
         <v>99</v>
@@ -5839,7 +5842,7 @@
         <v>22</v>
       </c>
       <c r="L76" s="16" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="M76" s="16" t="s">
         <v>24</v>
@@ -5853,10 +5856,10 @@
         <v>73</v>
       </c>
       <c r="B77" s="15" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C77" s="15" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D77" s="15" t="s">
         <v>52</v>
@@ -5880,10 +5883,10 @@
         <v>127</v>
       </c>
       <c r="K77" s="15" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="L77" s="16" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="M77" s="16" t="s">
         <v>24</v>
@@ -5897,10 +5900,10 @@
         <v>74</v>
       </c>
       <c r="B78" s="15" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C78" s="15" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D78" s="15" t="s">
         <v>52</v>
@@ -5924,10 +5927,10 @@
         <v>127</v>
       </c>
       <c r="K78" s="15" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L78" s="16" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="M78" s="16" t="s">
         <v>24</v>
@@ -5941,10 +5944,10 @@
         <v>75</v>
       </c>
       <c r="B79" s="15" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C79" s="15" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D79" s="15" t="s">
         <v>52</v>
@@ -5968,10 +5971,10 @@
         <v>127</v>
       </c>
       <c r="K79" s="15" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="L79" s="16" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="M79" s="16" t="s">
         <v>24</v>
@@ -5985,10 +5988,10 @@
         <v>76</v>
       </c>
       <c r="B80" s="15" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C80" s="15" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D80" s="15" t="s">
         <v>52</v>
@@ -6012,10 +6015,10 @@
         <v>127</v>
       </c>
       <c r="K80" s="15" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="L80" s="16" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="M80" s="16" t="s">
         <v>24</v>
@@ -6029,10 +6032,10 @@
         <v>77</v>
       </c>
       <c r="B81" s="15" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C81" s="15" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D81" s="15" t="s">
         <v>32</v>
@@ -6041,16 +6044,16 @@
         <v>41</v>
       </c>
       <c r="F81" s="15" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="G81" s="15" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="H81" s="15" t="s">
         <v>21</v>
       </c>
       <c r="I81" s="15" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="J81" s="15" t="s">
         <v>22</v>
@@ -6059,13 +6062,13 @@
         <v>22</v>
       </c>
       <c r="L81" s="16" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="M81" s="16" t="s">
         <v>24</v>
       </c>
       <c r="N81" s="16" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="82" ht="19" spans="1:14">
@@ -6073,19 +6076,19 @@
         <v>78</v>
       </c>
       <c r="B82" s="15" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C82" s="15" t="s">
-        <v>192</v>
+        <v>269</v>
       </c>
       <c r="D82" s="15" t="s">
-        <v>193</v>
+        <v>270</v>
       </c>
       <c r="E82" s="15" t="s">
         <v>22</v>
       </c>
       <c r="F82" s="15" t="s">
-        <v>194</v>
+        <v>271</v>
       </c>
       <c r="G82" s="15" t="s">
         <v>22</v>
@@ -6103,13 +6106,13 @@
         <v>22</v>
       </c>
       <c r="L82" s="16" t="s">
+        <v>272</v>
+      </c>
+      <c r="M82" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="N82" s="16" t="s">
         <v>195</v>
-      </c>
-      <c r="M82" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="N82" s="16" t="s">
-        <v>196</v>
       </c>
     </row>
   </sheetData>
@@ -6145,7 +6148,7 @@
   <sheetData>
     <row r="1" ht="62" customHeight="1" spans="1:8">
       <c r="A1" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -6157,25 +6160,25 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>14</v>
@@ -6183,28 +6186,28 @@
     </row>
     <row r="3" ht="34" customHeight="1" spans="1:8">
       <c r="A3" s="3" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="4" ht="34" customHeight="1" spans="1:8">
@@ -6212,65 +6215,65 @@
         <v>70</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>355</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>356</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>351</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>358</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1" spans="1:8">
       <c r="A5" s="3" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1" spans="1:8">
       <c r="A6" s="3" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>21</v>
@@ -6279,10 +6282,10 @@
         <v>24</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1" spans="1:8">
@@ -6290,25 +6293,25 @@
         <v>46</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1" spans="1:8">
@@ -6316,13 +6319,13 @@
         <v>92</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>21</v>
@@ -6331,10 +6334,10 @@
         <v>24</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:8">
@@ -6342,25 +6345,25 @@
         <v>60</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:8">
@@ -6368,39 +6371,39 @@
         <v>34</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1" spans="1:8">
       <c r="A11" s="3" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>21</v>
@@ -6409,10 +6412,10 @@
         <v>24</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1" spans="1:8">
@@ -6420,13 +6423,13 @@
         <v>19</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>21</v>
@@ -6435,10 +6438,10 @@
         <v>24</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1" spans="1:8">
@@ -6446,25 +6449,25 @@
         <v>154</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>24</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
     </row>
     <row r="14" ht="34" customHeight="1" spans="1:8">
@@ -6472,13 +6475,13 @@
         <v>53</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>21</v>
@@ -6487,24 +6490,24 @@
         <v>24</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="15" ht="34" customHeight="1" spans="1:8">
       <c r="A15" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>22</v>
@@ -6513,10 +6516,10 @@
         <v>24</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat:add code and qspi
</commit_message>
<xml_diff>
--- a/99_Doc/voice_checkpoint_resouce_map.xlsx
+++ b/99_Doc/voice_checkpoint_resouce_map.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="25550" windowHeight="13220"/>
+    <workbookView windowWidth="29360" windowHeight="13220" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="引脚分配" sheetId="1" r:id="rId1"/>
@@ -39,6 +39,11 @@
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1142" uniqueCount="421">
   <si>
     <r>
+      <rPr>
+        <sz val="72"/>
+        <rFont val="Carlito"/>
+        <charset val="134"/>
+      </rPr>
       <t>AT32F435VGT7 MCU</t>
     </r>
     <r>
@@ -1200,10 +1205,10 @@
     <t>PB1 SCK；PC11 CS；PA6/PA7/PC4/PC5 IO0~3</t>
   </si>
   <si>
-    <t>ClockDiv=3；Mode 0；XIP关闭</t>
-  </si>
-  <si>
-    <t>QSPI内部DMA阈值Word08</t>
+    <t>ClockDiv=12；Mode 0；XIP关闭CMD模式-在debug阶段我使用的分配是12，QSPI的主频是12Mhz,等待稳定后将会提高</t>
+  </si>
+  <si>
+    <t>QSPI内部DMA阈值Word08,但是没有显示的配置DMA或EDMA,调试阶段看波形</t>
   </si>
   <si>
     <t>数据源预留</t>
@@ -6248,7 +6253,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1" spans="1:8">
+    <row r="9" ht="43.5" spans="1:8">
       <c r="A9" s="3" t="s">
         <v>60</v>
       </c>

</xml_diff>

<commit_message>
feat: add USB Host FatFs read-write support and board tests
</commit_message>
<xml_diff>
--- a/99_Doc/voice_checkpoint_resouce_map.xlsx
+++ b/99_Doc/voice_checkpoint_resouce_map.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="23770" windowHeight="12620"/>
+    <workbookView windowWidth="26080" windowHeight="12620" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="引脚分配" sheetId="1" r:id="rId1"/>
@@ -1286,7 +1286,7 @@
     <t>USB内部</t>
   </si>
   <si>
-    <t>用途模式待上层USB功能确认</t>
+    <t>USB配合FATFS进行,U盘的读写,初步功能已经可以读写-&gt;USB升级还没实现.</t>
   </si>
   <si>
     <t>wk_usb_otgfs.c</t>

</xml_diff>